<commit_message>
Rebuild local SEO citation and outreach materials with real targets
- Add year founded (2013) and certifications to business profile
- Fill in Yelp year established, add missing Neustar Localeze entry
- Rewrite outreach drafts with 20 researched Austin targets:
  custom home builders (Sterling, Silverton, Nalle, Revent, Grand Endeavor),
  real estate blogs (Realty Austin, Bramlett Partners, CultureMap Austin),
  interior designers (Etch Design, Robin Bond, Amity Worrel),
  painters/roofers (21st Century, Five Star, RoofCrafters),
  suppliers (Mastercast, Sto Corp, Texas Stucco Supply, AHI, Longhorn)
- Add 10-week outreach sequencing plan prioritized by impact
- Regenerate tracker with all 18 directories including home services

Co-Authored-By: Claude Opus 4.6 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011wddH6XkXdgp69wu5Sr5hZ
</commit_message>
<xml_diff>
--- a/Local SEO/citation-tracker.xlsx
+++ b/Local SEO/citation-tracker.xlsx
@@ -435,7 +435,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I18"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="28" customWidth="1" min="1" max="1"/>
@@ -537,7 +537,7 @@
     <row r="4">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>Apple Business Connect</t>
+          <t>Apple Maps / Business Connect</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr"/>
@@ -632,7 +632,7 @@
     <row r="9">
       <c r="A9" s="2" t="inlineStr">
         <is>
-          <t>Yellow Pages</t>
+          <t>Neustar Localeze</t>
         </is>
       </c>
       <c r="B9" s="2" t="inlineStr"/>
@@ -651,7 +651,7 @@
     <row r="10">
       <c r="A10" s="2" t="inlineStr">
         <is>
-          <t>Better Business Bureau</t>
+          <t>Yellow Pages</t>
         </is>
       </c>
       <c r="B10" s="2" t="inlineStr"/>
@@ -670,7 +670,7 @@
     <row r="11">
       <c r="A11" s="2" t="inlineStr">
         <is>
-          <t>Nextdoor Business</t>
+          <t>Better Business Bureau</t>
         </is>
       </c>
       <c r="B11" s="2" t="inlineStr"/>
@@ -689,7 +689,7 @@
     <row r="12">
       <c r="A12" s="2" t="inlineStr">
         <is>
-          <t>Manta</t>
+          <t>Nextdoor Business</t>
         </is>
       </c>
       <c r="B12" s="2" t="inlineStr"/>
@@ -708,7 +708,7 @@
     <row r="13">
       <c r="A13" s="2" t="inlineStr">
         <is>
-          <t>Austin Chamber of Commerce</t>
+          <t>Manta</t>
         </is>
       </c>
       <c r="B13" s="2" t="inlineStr"/>
@@ -727,7 +727,7 @@
     <row r="14">
       <c r="A14" s="2" t="inlineStr">
         <is>
-          <t>Angi</t>
+          <t>Austin Chamber of Commerce</t>
         </is>
       </c>
       <c r="B14" s="2" t="inlineStr"/>
@@ -746,7 +746,7 @@
     <row r="15">
       <c r="A15" s="2" t="inlineStr">
         <is>
-          <t>HomeAdvisor</t>
+          <t>Angi</t>
         </is>
       </c>
       <c r="B15" s="2" t="inlineStr"/>
@@ -765,7 +765,7 @@
     <row r="16">
       <c r="A16" s="2" t="inlineStr">
         <is>
-          <t>Thumbtack</t>
+          <t>HomeAdvisor</t>
         </is>
       </c>
       <c r="B16" s="2" t="inlineStr"/>
@@ -784,7 +784,7 @@
     <row r="17">
       <c r="A17" s="2" t="inlineStr">
         <is>
-          <t>Houzz</t>
+          <t>Thumbtack</t>
         </is>
       </c>
       <c r="B17" s="2" t="inlineStr"/>
@@ -803,7 +803,7 @@
     <row r="18">
       <c r="A18" s="2" t="inlineStr">
         <is>
-          <t>MapQuest</t>
+          <t>Houzz</t>
         </is>
       </c>
       <c r="B18" s="2" t="inlineStr"/>
@@ -818,6 +818,25 @@
       <c r="G18" s="2" t="inlineStr"/>
       <c r="H18" s="2" t="inlineStr"/>
       <c r="I18" s="2" t="inlineStr"/>
+    </row>
+    <row r="19">
+      <c r="A19" s="2" t="inlineStr">
+        <is>
+          <t>MapQuest</t>
+        </is>
+      </c>
+      <c r="B19" s="2" t="inlineStr"/>
+      <c r="C19" s="2" t="inlineStr"/>
+      <c r="D19" s="2" t="inlineStr">
+        <is>
+          <t>Not Started</t>
+        </is>
+      </c>
+      <c r="E19" s="2" t="inlineStr"/>
+      <c r="F19" s="2" t="inlineStr"/>
+      <c r="G19" s="2" t="inlineStr"/>
+      <c r="H19" s="2" t="inlineStr"/>
+      <c r="I19" s="2" t="inlineStr"/>
     </row>
   </sheetData>
   <dataValidations count="2">

</xml_diff>